<commit_message>
Add configurable routing overrides
</commit_message>
<xml_diff>
--- a/templates/sorting_configuration.xlsx
+++ b/templates/sorting_configuration.xlsx
@@ -8,18 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\jcs507\workspace\pgl\sorting\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0580B20A-B6D1-46CB-8F06-271F5AE608D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AB106A6-B091-4BDD-A3D3-1F103BE05049}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4820" yWindow="3090" windowWidth="19200" windowHeight="11170" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
     <sheet name="Pathologists" sheetId="2" r:id="rId2"/>
     <sheet name="CaseTypes" sheetId="3" r:id="rId3"/>
     <sheet name="AssignmentSettings" sheetId="7" r:id="rId4"/>
-    <sheet name="Prefixes" sheetId="4" r:id="rId5"/>
-    <sheet name="Hospitals" sheetId="5" r:id="rId6"/>
-    <sheet name="Lists" sheetId="6" state="hidden" r:id="rId7"/>
+    <sheet name="RoutingOverrides" sheetId="8" r:id="rId5"/>
+    <sheet name="Prefixes" sheetId="4" r:id="rId6"/>
+    <sheet name="Hospitals" sheetId="5" r:id="rId7"/>
+    <sheet name="Lists" sheetId="6" state="hidden" r:id="rId8"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -206,7 +207,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="258">
   <si>
     <t>PGL Sorting Engine — Configuration Workbook</t>
   </si>
@@ -905,13 +906,88 @@
   </si>
   <si>
     <t>wh_starting_weight</t>
+  </si>
+  <si>
+    <t>rule_name</t>
+  </si>
+  <si>
+    <t>routing_mode</t>
+  </si>
+  <si>
+    <t>destination_location</t>
+  </si>
+  <si>
+    <t>required_subspecialty</t>
+  </si>
+  <si>
+    <t>OL-BX to OLOL</t>
+  </si>
+  <si>
+    <t>always_required</t>
+  </si>
+  <si>
+    <t>OL-SC to OLOL</t>
+  </si>
+  <si>
+    <t>OL-SG to OLOL</t>
+  </si>
+  <si>
+    <t>BB-BX to BRG</t>
+  </si>
+  <si>
+    <t>BB-SC to BRG</t>
+  </si>
+  <si>
+    <t>BB-SG to BRG</t>
+  </si>
+  <si>
+    <t>PG-GI Lane to MET</t>
+  </si>
+  <si>
+    <t>LANE RMC</t>
+  </si>
+  <si>
+    <t>preferred_until_target</t>
+  </si>
+  <si>
+    <t>OUR LADY OF THE LAKE ASCENSION</t>
+  </si>
+  <si>
+    <t>PG-GI Asc to OLOL</t>
+  </si>
+  <si>
+    <t>required_if_subspecialist_present</t>
+  </si>
+  <si>
+    <t>BB-CP to BRG</t>
+  </si>
+  <si>
+    <t>OLOL CHILDREN'S HOSPITAL</t>
+  </si>
+  <si>
+    <t>OL-GP CH to SG</t>
+  </si>
+  <si>
+    <t>HP;BM;GP</t>
+  </si>
+  <si>
+    <t>BATON ROUGE GENERAL BLUEBONNET</t>
+  </si>
+  <si>
+    <t>identify_only</t>
+  </si>
+  <si>
+    <t>PG-BO recenter identify</t>
+  </si>
+  <si>
+    <t>RECENTER</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -939,6 +1015,18 @@
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
@@ -1039,7 +1127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -1060,18 +1148,28 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1438,10 +1536,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9"/>
+      <c r="B1" s="17"/>
     </row>
     <row r="3" spans="1:2" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
@@ -1607,7 +1705,7 @@
         <v>201</v>
       </c>
       <c r="C7" t="s">
-        <v>198</v>
+        <v>253</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
@@ -1994,18 +2092,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="10" t="s">
         <v>231</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="11" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" s="10">
+      <c r="A2" s="8">
         <v>200</v>
       </c>
-      <c r="B2" s="11">
+      <c r="B2" s="9">
         <v>400</v>
       </c>
     </row>
@@ -2015,6 +2113,272 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{315E4CB5-22C5-4E47-AA3D-EAA24DD07D5A}">
+  <sheetPr>
+    <tabColor rgb="FFFFFF00"/>
+  </sheetPr>
+  <dimension ref="A1:L12"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="19.36328125" customWidth="1"/>
+    <col min="2" max="2" width="31" customWidth="1"/>
+    <col min="4" max="4" width="9.7265625" customWidth="1"/>
+    <col min="5" max="5" width="30.54296875" customWidth="1"/>
+    <col min="6" max="6" width="19.26953125" customWidth="1"/>
+    <col min="7" max="7" width="17.1796875" customWidth="1"/>
+    <col min="8" max="8" width="19.54296875" customWidth="1"/>
+    <col min="9" max="12" width="8.7265625" style="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A1" s="10" t="s">
+        <v>233</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>234</v>
+      </c>
+      <c r="F1" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1" s="11" t="s">
+        <v>236</v>
+      </c>
+      <c r="I1" s="12"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="13"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>237</v>
+      </c>
+      <c r="C2" t="s">
+        <v>186</v>
+      </c>
+      <c r="D2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E2" t="s">
+        <v>238</v>
+      </c>
+      <c r="F2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>239</v>
+      </c>
+      <c r="C3" t="s">
+        <v>186</v>
+      </c>
+      <c r="D3" t="s">
+        <v>59</v>
+      </c>
+      <c r="E3" t="s">
+        <v>238</v>
+      </c>
+      <c r="F3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>240</v>
+      </c>
+      <c r="C4" t="s">
+        <v>186</v>
+      </c>
+      <c r="D4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E4" t="s">
+        <v>238</v>
+      </c>
+      <c r="F4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>241</v>
+      </c>
+      <c r="C5" t="s">
+        <v>41</v>
+      </c>
+      <c r="D5" t="s">
+        <v>45</v>
+      </c>
+      <c r="E5" t="s">
+        <v>238</v>
+      </c>
+      <c r="F5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>242</v>
+      </c>
+      <c r="C6" t="s">
+        <v>41</v>
+      </c>
+      <c r="D6" t="s">
+        <v>59</v>
+      </c>
+      <c r="E6" t="s">
+        <v>238</v>
+      </c>
+      <c r="F6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>243</v>
+      </c>
+      <c r="C7" t="s">
+        <v>41</v>
+      </c>
+      <c r="D7" t="s">
+        <v>60</v>
+      </c>
+      <c r="E7" t="s">
+        <v>238</v>
+      </c>
+      <c r="F7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>244</v>
+      </c>
+      <c r="B8" t="s">
+        <v>245</v>
+      </c>
+      <c r="C8" t="s">
+        <v>187</v>
+      </c>
+      <c r="D8" t="s">
+        <v>51</v>
+      </c>
+      <c r="E8" t="s">
+        <v>246</v>
+      </c>
+      <c r="F8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>248</v>
+      </c>
+      <c r="B9" t="s">
+        <v>247</v>
+      </c>
+      <c r="C9" t="s">
+        <v>187</v>
+      </c>
+      <c r="D9" t="s">
+        <v>51</v>
+      </c>
+      <c r="E9" t="s">
+        <v>35</v>
+      </c>
+      <c r="G9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>250</v>
+      </c>
+      <c r="B10" s="15" t="s">
+        <v>254</v>
+      </c>
+      <c r="C10" t="s">
+        <v>41</v>
+      </c>
+      <c r="D10" t="s">
+        <v>46</v>
+      </c>
+      <c r="E10" t="s">
+        <v>249</v>
+      </c>
+      <c r="F10" t="s">
+        <v>34</v>
+      </c>
+      <c r="H10" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>252</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>251</v>
+      </c>
+      <c r="C11" t="s">
+        <v>186</v>
+      </c>
+      <c r="D11" t="s">
+        <v>52</v>
+      </c>
+      <c r="E11" t="s">
+        <v>249</v>
+      </c>
+      <c r="F11" t="s">
+        <v>32</v>
+      </c>
+      <c r="H11" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>256</v>
+      </c>
+      <c r="B12" t="s">
+        <v>257</v>
+      </c>
+      <c r="C12" t="s">
+        <v>187</v>
+      </c>
+      <c r="D12" t="s">
+        <v>43</v>
+      </c>
+      <c r="E12" t="s">
+        <v>255</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E150" xr:uid="{D496C206-4DA8-4436-80F0-5B68453E1DB3}">
+      <formula1>"identify_only,always_required,required_if_subspecialist_present,preferred,preferred_until_target"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F150" xr:uid="{F71E1F24-18D5-4528-99BF-60F86FFB176D}">
+      <formula1>"OLOL,BRG,WH,MET,TEXAS,OMEGA"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <tabColor rgb="FFED7D31"/>
@@ -2116,7 +2480,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr>
     <tabColor rgb="FFA5A5A5"/>
@@ -3105,7 +3469,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>

<commit_message>
Add routing weight caps and complete distribution grids
</commit_message>
<xml_diff>
--- a/templates/sorting_configuration.xlsx
+++ b/templates/sorting_configuration.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\jcs507\workspace\pgl\sorting\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AB106A6-B091-4BDD-A3D3-1F103BE05049}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{090C8B18-4758-4304-8FDB-049E42DBCE55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -207,7 +207,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="258">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="264">
   <si>
     <t>PGL Sorting Engine — Configuration Workbook</t>
   </si>
@@ -971,9 +971,6 @@
     <t>HP;BM;GP</t>
   </si>
   <si>
-    <t>BATON ROUGE GENERAL BLUEBONNET</t>
-  </si>
-  <si>
     <t>identify_only</t>
   </si>
   <si>
@@ -981,6 +978,27 @@
   </si>
   <si>
     <t>RECENTER</t>
+  </si>
+  <si>
+    <t>weight_cap</t>
+  </si>
+  <si>
+    <t>preferred_until_weight_cap</t>
+  </si>
+  <si>
+    <t>OL-PB to Met preferred</t>
+  </si>
+  <si>
+    <t>BB-PB to Met preferred</t>
+  </si>
+  <si>
+    <t>PG-PB to Met preferred</t>
+  </si>
+  <si>
+    <t>OL-CP to OLOL</t>
+  </si>
+  <si>
+    <t>OL-CY to OLOL</t>
   </si>
 </sst>
 </file>
@@ -2117,17 +2135,18 @@
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.36328125" customWidth="1"/>
+    <col min="1" max="1" width="21.90625" customWidth="1"/>
     <col min="2" max="2" width="31" customWidth="1"/>
     <col min="4" max="4" width="9.7265625" customWidth="1"/>
     <col min="5" max="5" width="30.54296875" customWidth="1"/>
     <col min="6" max="6" width="19.26953125" customWidth="1"/>
     <col min="7" max="7" width="17.1796875" customWidth="1"/>
     <col min="8" max="8" width="19.54296875" customWidth="1"/>
-    <col min="9" max="12" width="8.7265625" style="14"/>
+    <col min="9" max="9" width="12" style="14" customWidth="1"/>
+    <col min="10" max="12" width="8.7265625" style="14"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.35">
@@ -2155,7 +2174,9 @@
       <c r="H1" s="11" t="s">
         <v>236</v>
       </c>
-      <c r="I1" s="12"/>
+      <c r="I1" s="11" t="s">
+        <v>257</v>
+      </c>
       <c r="J1" s="13"/>
       <c r="K1" s="12"/>
       <c r="L1" s="13"/>
@@ -2302,13 +2323,11 @@
         <v>32</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>250</v>
       </c>
-      <c r="B10" s="15" t="s">
-        <v>254</v>
-      </c>
+      <c r="B10" s="15"/>
       <c r="C10" t="s">
         <v>41</v>
       </c>
@@ -2350,10 +2369,10 @@
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
+        <v>255</v>
+      </c>
+      <c r="B12" t="s">
         <v>256</v>
-      </c>
-      <c r="B12" t="s">
-        <v>257</v>
       </c>
       <c r="C12" t="s">
         <v>187</v>
@@ -2362,13 +2381,113 @@
         <v>43</v>
       </c>
       <c r="E12" t="s">
-        <v>255</v>
+        <v>254</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>259</v>
+      </c>
+      <c r="C13" t="s">
+        <v>186</v>
+      </c>
+      <c r="D13" t="s">
+        <v>57</v>
+      </c>
+      <c r="E13" t="s">
+        <v>258</v>
+      </c>
+      <c r="F13" t="s">
+        <v>38</v>
+      </c>
+      <c r="I13" s="14">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>260</v>
+      </c>
+      <c r="C14" t="s">
+        <v>41</v>
+      </c>
+      <c r="D14" t="s">
+        <v>57</v>
+      </c>
+      <c r="E14" t="s">
+        <v>258</v>
+      </c>
+      <c r="F14" t="s">
+        <v>38</v>
+      </c>
+      <c r="I14" s="14">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>261</v>
+      </c>
+      <c r="C15" t="s">
+        <v>187</v>
+      </c>
+      <c r="D15" t="s">
+        <v>57</v>
+      </c>
+      <c r="E15" t="s">
+        <v>258</v>
+      </c>
+      <c r="F15" t="s">
+        <v>38</v>
+      </c>
+      <c r="I15" s="14">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>262</v>
+      </c>
+      <c r="C16" t="s">
+        <v>186</v>
+      </c>
+      <c r="D16" t="s">
+        <v>46</v>
+      </c>
+      <c r="E16" t="s">
+        <v>249</v>
+      </c>
+      <c r="F16" t="s">
+        <v>32</v>
+      </c>
+      <c r="H16" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>263</v>
+      </c>
+      <c r="C17" t="s">
+        <v>186</v>
+      </c>
+      <c r="D17" t="s">
+        <v>47</v>
+      </c>
+      <c r="E17" t="s">
+        <v>249</v>
+      </c>
+      <c r="F17" t="s">
+        <v>32</v>
+      </c>
+      <c r="H17" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E150" xr:uid="{D496C206-4DA8-4436-80F0-5B68453E1DB3}">
-      <formula1>"identify_only,always_required,required_if_subspecialist_present,preferred,preferred_until_target"</formula1>
+      <formula1>"identify_only,always_required,required_if_subspecialist_present,preferred,preferred_until_target,preferred_until_weight_cap"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F150" xr:uid="{F71E1F24-18D5-4528-99BF-60F86FFB176D}">
       <formula1>"OLOL,BRG,WH,MET,TEXAS,OMEGA"</formula1>

</xml_diff>

<commit_message>
Add Tkinter desktop interface
</commit_message>
<xml_diff>
--- a/templates/sorting_configuration.xlsx
+++ b/templates/sorting_configuration.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\jcs507\workspace\pgl\sorting\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{090C8B18-4758-4304-8FDB-049E42DBCE55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6C220C5-345F-471D-9B75-3809B8C65ABC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -207,7 +207,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="583" uniqueCount="282">
   <si>
     <t>PGL Sorting Engine — Configuration Workbook</t>
   </si>
@@ -999,6 +999,60 @@
   </si>
   <si>
     <t>OL-CY to OLOL</t>
+  </si>
+  <si>
+    <t>OL-DA to OLOL</t>
+  </si>
+  <si>
+    <t>OL-HM to OLOL</t>
+  </si>
+  <si>
+    <t>OL-NP to OLOL</t>
+  </si>
+  <si>
+    <t>OL-RF to OLOL</t>
+  </si>
+  <si>
+    <t>PG-RF to OLOL</t>
+  </si>
+  <si>
+    <t>PG-HM to OLOL</t>
+  </si>
+  <si>
+    <t>BB-BO to BRG</t>
+  </si>
+  <si>
+    <t>BB-BR to BRG</t>
+  </si>
+  <si>
+    <t>BB-DA to BRG</t>
+  </si>
+  <si>
+    <t>BB-NP to BRG</t>
+  </si>
+  <si>
+    <t>PG-GI Angels to OLOL</t>
+  </si>
+  <si>
+    <t>OL-GI to OLOL</t>
+  </si>
+  <si>
+    <t>BB-GI to BRG</t>
+  </si>
+  <si>
+    <t>BB-GU to BRG</t>
+  </si>
+  <si>
+    <t>LU-BX to OLOL</t>
+  </si>
+  <si>
+    <t>PG-BO to BRG or WH</t>
+  </si>
+  <si>
+    <t>BRG; WH</t>
+  </si>
+  <si>
+    <t>PG-SG to MET</t>
   </si>
 </sst>
 </file>
@@ -1145,7 +1199,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -1183,6 +1237,9 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1554,10 +1611,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="17"/>
+      <c r="B1" s="18"/>
     </row>
     <row r="3" spans="1:2" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
@@ -2135,7 +2192,7 @@
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21.90625" customWidth="1"/>
@@ -2234,262 +2291,554 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>241</v>
+        <v>264</v>
       </c>
       <c r="C5" t="s">
-        <v>41</v>
+        <v>186</v>
       </c>
       <c r="D5" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="E5" t="s">
         <v>238</v>
       </c>
       <c r="F5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>242</v>
+        <v>265</v>
       </c>
       <c r="C6" t="s">
-        <v>41</v>
+        <v>186</v>
       </c>
       <c r="D6" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="E6" t="s">
         <v>238</v>
       </c>
       <c r="F6" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>243</v>
+        <v>266</v>
       </c>
       <c r="C7" t="s">
-        <v>41</v>
+        <v>186</v>
       </c>
       <c r="D7" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="E7" t="s">
         <v>238</v>
       </c>
       <c r="F7" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>244</v>
-      </c>
-      <c r="B8" t="s">
-        <v>245</v>
+        <v>267</v>
       </c>
       <c r="C8" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D8" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="E8" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
       <c r="F8" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>248</v>
-      </c>
-      <c r="B9" t="s">
-        <v>247</v>
+        <v>275</v>
       </c>
       <c r="C9" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D9" t="s">
         <v>51</v>
       </c>
       <c r="E9" t="s">
-        <v>35</v>
-      </c>
-      <c r="G9" t="s">
+        <v>238</v>
+      </c>
+      <c r="F9" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>250</v>
-      </c>
-      <c r="B10" s="15"/>
+        <v>268</v>
+      </c>
       <c r="C10" t="s">
-        <v>41</v>
+        <v>187</v>
       </c>
       <c r="D10" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="E10" t="s">
-        <v>249</v>
+        <v>238</v>
       </c>
       <c r="F10" t="s">
-        <v>34</v>
-      </c>
-      <c r="H10" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>252</v>
-      </c>
-      <c r="B11" s="15" t="s">
-        <v>251</v>
+        <v>269</v>
       </c>
       <c r="C11" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D11" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E11" t="s">
-        <v>249</v>
+        <v>238</v>
       </c>
       <c r="F11" t="s">
         <v>32</v>
       </c>
-      <c r="H11" t="s">
-        <v>52</v>
-      </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>255</v>
-      </c>
-      <c r="B12" t="s">
-        <v>256</v>
+        <v>278</v>
       </c>
       <c r="C12" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D12" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E12" t="s">
-        <v>254</v>
+        <v>238</v>
+      </c>
+      <c r="F12" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>259</v>
+        <v>241</v>
       </c>
       <c r="C13" t="s">
-        <v>186</v>
+        <v>41</v>
       </c>
       <c r="D13" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="E13" t="s">
-        <v>258</v>
+        <v>238</v>
       </c>
       <c r="F13" t="s">
-        <v>38</v>
-      </c>
-      <c r="I13" s="14">
-        <v>160</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>260</v>
+        <v>242</v>
       </c>
       <c r="C14" t="s">
         <v>41</v>
       </c>
       <c r="D14" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E14" t="s">
-        <v>258</v>
+        <v>238</v>
       </c>
       <c r="F14" t="s">
-        <v>38</v>
-      </c>
-      <c r="I14" s="14">
-        <v>160</v>
+        <v>34</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>261</v>
+        <v>243</v>
       </c>
       <c r="C15" t="s">
-        <v>187</v>
+        <v>41</v>
       </c>
       <c r="D15" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E15" t="s">
-        <v>258</v>
+        <v>238</v>
       </c>
       <c r="F15" t="s">
-        <v>38</v>
-      </c>
-      <c r="I15" s="14">
-        <v>160</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
       <c r="C16" t="s">
-        <v>186</v>
+        <v>41</v>
       </c>
       <c r="D16" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E16" t="s">
-        <v>249</v>
+        <v>238</v>
       </c>
       <c r="F16" t="s">
-        <v>32</v>
-      </c>
-      <c r="H16" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
+        <v>271</v>
+      </c>
+      <c r="C17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D17" t="s">
+        <v>44</v>
+      </c>
+      <c r="E17" t="s">
+        <v>238</v>
+      </c>
+      <c r="F17" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>272</v>
+      </c>
+      <c r="C18" t="s">
+        <v>41</v>
+      </c>
+      <c r="D18" t="s">
+        <v>48</v>
+      </c>
+      <c r="E18" t="s">
+        <v>238</v>
+      </c>
+      <c r="F18" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>273</v>
+      </c>
+      <c r="C19" t="s">
+        <v>41</v>
+      </c>
+      <c r="D19" t="s">
+        <v>56</v>
+      </c>
+      <c r="E19" t="s">
+        <v>238</v>
+      </c>
+      <c r="F19" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>276</v>
+      </c>
+      <c r="C20" t="s">
+        <v>41</v>
+      </c>
+      <c r="D20" t="s">
+        <v>51</v>
+      </c>
+      <c r="E20" t="s">
+        <v>238</v>
+      </c>
+      <c r="F20" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>277</v>
+      </c>
+      <c r="C21" t="s">
+        <v>41</v>
+      </c>
+      <c r="D21" t="s">
+        <v>53</v>
+      </c>
+      <c r="E21" t="s">
+        <v>238</v>
+      </c>
+      <c r="F21" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>248</v>
+      </c>
+      <c r="B22" t="s">
+        <v>247</v>
+      </c>
+      <c r="C22" t="s">
+        <v>187</v>
+      </c>
+      <c r="D22" t="s">
+        <v>51</v>
+      </c>
+      <c r="E22" t="s">
+        <v>35</v>
+      </c>
+      <c r="G22" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>274</v>
+      </c>
+      <c r="B23" s="16" t="s">
+        <v>158</v>
+      </c>
+      <c r="C23" t="s">
+        <v>187</v>
+      </c>
+      <c r="D23" t="s">
+        <v>51</v>
+      </c>
+      <c r="E23" t="s">
+        <v>35</v>
+      </c>
+      <c r="G23" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>279</v>
+      </c>
+      <c r="C24" t="s">
+        <v>187</v>
+      </c>
+      <c r="D24" t="s">
+        <v>43</v>
+      </c>
+      <c r="E24" t="s">
+        <v>35</v>
+      </c>
+      <c r="G24" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>281</v>
+      </c>
+      <c r="C25" t="s">
+        <v>187</v>
+      </c>
+      <c r="D25" t="s">
+        <v>60</v>
+      </c>
+      <c r="E25" t="s">
+        <v>35</v>
+      </c>
+      <c r="G25" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>244</v>
+      </c>
+      <c r="B28" t="s">
+        <v>245</v>
+      </c>
+      <c r="C28" t="s">
+        <v>187</v>
+      </c>
+      <c r="D28" t="s">
+        <v>51</v>
+      </c>
+      <c r="E28" t="s">
+        <v>246</v>
+      </c>
+      <c r="F28" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>250</v>
+      </c>
+      <c r="B30" s="15"/>
+      <c r="C30" t="s">
+        <v>41</v>
+      </c>
+      <c r="D30" t="s">
+        <v>46</v>
+      </c>
+      <c r="E30" t="s">
+        <v>249</v>
+      </c>
+      <c r="F30" t="s">
+        <v>34</v>
+      </c>
+      <c r="H30" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>252</v>
+      </c>
+      <c r="B31" s="15" t="s">
+        <v>251</v>
+      </c>
+      <c r="C31" t="s">
+        <v>186</v>
+      </c>
+      <c r="D31" t="s">
+        <v>52</v>
+      </c>
+      <c r="E31" t="s">
+        <v>249</v>
+      </c>
+      <c r="F31" t="s">
+        <v>32</v>
+      </c>
+      <c r="H31" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>255</v>
+      </c>
+      <c r="B32" t="s">
+        <v>256</v>
+      </c>
+      <c r="C32" t="s">
+        <v>187</v>
+      </c>
+      <c r="D32" t="s">
+        <v>43</v>
+      </c>
+      <c r="E32" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>259</v>
+      </c>
+      <c r="C33" t="s">
+        <v>186</v>
+      </c>
+      <c r="D33" t="s">
+        <v>57</v>
+      </c>
+      <c r="E33" t="s">
+        <v>258</v>
+      </c>
+      <c r="F33" t="s">
+        <v>38</v>
+      </c>
+      <c r="I33" s="14">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>260</v>
+      </c>
+      <c r="C34" t="s">
+        <v>41</v>
+      </c>
+      <c r="D34" t="s">
+        <v>57</v>
+      </c>
+      <c r="E34" t="s">
+        <v>258</v>
+      </c>
+      <c r="F34" t="s">
+        <v>38</v>
+      </c>
+      <c r="I34" s="14">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>261</v>
+      </c>
+      <c r="C35" t="s">
+        <v>187</v>
+      </c>
+      <c r="D35" t="s">
+        <v>57</v>
+      </c>
+      <c r="E35" t="s">
+        <v>258</v>
+      </c>
+      <c r="F35" t="s">
+        <v>38</v>
+      </c>
+      <c r="I35" s="14">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>262</v>
+      </c>
+      <c r="C36" t="s">
+        <v>186</v>
+      </c>
+      <c r="D36" t="s">
+        <v>46</v>
+      </c>
+      <c r="E36" t="s">
+        <v>249</v>
+      </c>
+      <c r="F36" t="s">
+        <v>32</v>
+      </c>
+      <c r="H36" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
         <v>263</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C37" t="s">
         <v>186</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D37" t="s">
         <v>47</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E37" t="s">
         <v>249</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F37" t="s">
         <v>32</v>
       </c>
-      <c r="H17" t="s">
+      <c r="H37" t="s">
         <v>47</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E150" xr:uid="{D496C206-4DA8-4436-80F0-5B68453E1DB3}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E28 E30:E150 E2:E24" xr:uid="{D496C206-4DA8-4436-80F0-5B68453E1DB3}">
       <formula1>"identify_only,always_required,required_if_subspecialist_present,preferred,preferred_until_target,preferred_until_weight_cap"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F150" xr:uid="{F71E1F24-18D5-4528-99BF-60F86FFB176D}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F28 F30:F150 F2:F24" xr:uid="{F71E1F24-18D5-4528-99BF-60F86FFB176D}">
       <formula1>"OLOL,BRG,WH,MET,TEXAS,OMEGA"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>